<commit_message>
chore: update results.xlsx with new data
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,17 +434,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Model A (Full FT)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Model B (LoRA)</t>
         </is>
@@ -646,37 +658,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Accuracy</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Macro-F1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Precision Macro</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Recall Macro</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Invalid output rate</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Inference sec / 100</t>
         </is>
@@ -768,33 +780,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>BLEU</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>chrF</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Average output length (words)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Inference sec / 100</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Error example (worst case)</t>
         </is>
       </c>
     </row>
@@ -816,6 +833,11 @@
       <c r="E2" t="n">
         <v>7.6</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>'Exactly so,' said the Hatter: 'as the things get used up.' -&gt; '-' (gold: '« Justement, » dit le Chapelier, « à mesure que les tasses ont servi. »')</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -835,6 +857,11 @@
       <c r="E3" t="n">
         <v>8.199999999999999</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>"Coral insects," replied Cyrus Harding. -&gt; '--' (gold: '-- Les infusoires du corail, répondit Cyrus Smith.')</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -854,6 +881,7 @@
       <c r="E4" t="n">
         <v>0.6</v>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -866,38 +894,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Exact Match</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Token F1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Average answer length (words)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Average gold length (words)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Inference sec / 100</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Error example (worst case)</t>
         </is>
       </c>
     </row>
@@ -922,6 +955,11 @@
       <c r="F2" t="n">
         <v>2.8</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>How often are elections held for the Victorian Parliament? -&gt; 'annually' (gold: 'every four years')</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -944,6 +982,11 @@
       <c r="F3" t="n">
         <v>3.1</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>How often are elections held for the Victorian Parliament? -&gt; 'annually' (gold: 'every four years')</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -966,6 +1009,7 @@
       <c r="F4" t="n">
         <v>0.3</v>
       </c>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -982,37 +1026,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Classification score</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Translation score</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>QA score</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Overall score</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Train time (min)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Inference time / 100 examples (sec)</t>
         </is>
@@ -1108,37 +1152,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Row</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Gold answer</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Model A output</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Model B output</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>

</xml_diff>